<commit_message>
Written Smoke & Regression TCs
</commit_message>
<xml_diff>
--- a/test-output/CreatedUsers.xlsx
+++ b/test-output/CreatedUsers.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="122">
   <si>
     <t>First Name</t>
   </si>
@@ -284,6 +284,108 @@
   </si>
   <si>
     <t>SeleniumUser.4c504@infor.com</t>
+  </si>
+  <si>
+    <t>d6614</t>
+  </si>
+  <si>
+    <t>SeleniumUser.d6614@infor.com</t>
+  </si>
+  <si>
+    <t>67643</t>
+  </si>
+  <si>
+    <t>SeleniumUser.67643@infor.com</t>
+  </si>
+  <si>
+    <t>93f81</t>
+  </si>
+  <si>
+    <t>SeleniumUser.93f81@infor.com</t>
+  </si>
+  <si>
+    <t>dddc7</t>
+  </si>
+  <si>
+    <t>SeleniumUser.dddc7@infor.com</t>
+  </si>
+  <si>
+    <t>fcf14</t>
+  </si>
+  <si>
+    <t>SeleniumUser.fcf14@infor.com</t>
+  </si>
+  <si>
+    <t>7179e</t>
+  </si>
+  <si>
+    <t>SeleniumUser.7179e@infor.com</t>
+  </si>
+  <si>
+    <t>20afc</t>
+  </si>
+  <si>
+    <t>SeleniumUser.20afc@infor.com</t>
+  </si>
+  <si>
+    <t>9681f</t>
+  </si>
+  <si>
+    <t>SeleniumUser.9681f@infor.com</t>
+  </si>
+  <si>
+    <t>2450f</t>
+  </si>
+  <si>
+    <t>SeleniumUser.2450f@infor.com</t>
+  </si>
+  <si>
+    <t>9f589</t>
+  </si>
+  <si>
+    <t>SeleniumUser.9f589@infor.com</t>
+  </si>
+  <si>
+    <t>9b357</t>
+  </si>
+  <si>
+    <t>SeleniumUser.9b357@infor.com</t>
+  </si>
+  <si>
+    <t>b4e60</t>
+  </si>
+  <si>
+    <t>SeleniumUser.b4e60@infor.com</t>
+  </si>
+  <si>
+    <t>c7958</t>
+  </si>
+  <si>
+    <t>SeleniumUser.c7958@infor.com</t>
+  </si>
+  <si>
+    <t>dd58f</t>
+  </si>
+  <si>
+    <t>SeleniumUser.dd58f@infor.com</t>
+  </si>
+  <si>
+    <t>bf486</t>
+  </si>
+  <si>
+    <t>SeleniumUser.bf486@infor.com</t>
+  </si>
+  <si>
+    <t>42f71</t>
+  </si>
+  <si>
+    <t>SeleniumUser.42f71@infor.com</t>
+  </si>
+  <si>
+    <t>d8d24</t>
+  </si>
+  <si>
+    <t>SeleniumUser.d8d24@infor.com</t>
   </si>
 </sst>
 </file>
@@ -666,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="12.4453125"/>
@@ -1147,6 +1249,193 @@
         <v>87</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="C44" t="s" s="0">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="C45" t="s" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="C46" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="C47" t="s" s="0">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="C48" t="s" s="0">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="C49" t="s" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C50" t="s" s="0">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C51" t="s" s="0">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C52" t="s" s="0">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C53" t="s" s="0">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="C54" t="s" s="0">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="C55" t="s" s="0">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>112</v>
+      </c>
+      <c r="C56" t="s" s="0">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="C57" t="s" s="0">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="C58" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="C59" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="C60" t="s" s="0">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>